<commit_message>
Fix issue with Controlled Unit having IsImplantAttempt=true. Add support for showing counter desc. Support hot keys
</commit_message>
<xml_diff>
--- a/DesignDocs/Events.xlsx
+++ b/DesignDocs/Events.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstewa01\source\repos\happysulla\TheyveInvadedPleasantville\DesignDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EE4854B9-3660-4CDE-A10A-4EBC7F3F007D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{332CFE25-C099-4B4E-90C2-6D8A6D07304A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5700" yWindow="2355" windowWidth="21600" windowHeight="11145" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
+    <workbookView xWindow="28680" yWindow="90" windowWidth="29040" windowHeight="15510" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
   </bookViews>
   <sheets>
     <sheet name="Events" sheetId="1" r:id="rId1"/>
@@ -243,16 +243,6 @@
                                         &lt;InlineUIContainer&gt;&lt;Image Name='Continue011t' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
   </si>
   <si>
-    <t>&lt;Bold&gt;e013t Implant Removals&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r8.7.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; 
-&lt;InlineUIContainer&gt;&lt;Button Content='Implant Removal' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-The Town player may try to remove this implant from a defeated Alien controlled townsperson, thus breaking the Alien player's control.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
- Removing the implant generates an electric shock may erases all memory of the Alien HQ from the victim's memory, a unique safegard which is built into the implant's circuits.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Click a flashing space to begin.</t>
-  </si>
-  <si>
     <t>&lt;Bold&gt;e005 Random Movement&lt;/Bold&gt; &lt;InlineUIContainer&gt;&lt;Button Content='r6.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
 Four townspeople move randomly in any given turn. The &lt;InlineUIContainer&gt;&lt;Button Content='Townspeople' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table determines who moves. The destination is per the 
@@ -367,9 +357,21 @@
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;</t>
   </si>
   <si>
+    <t>&lt;Bold&gt;e013t Implant Removals&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r8.7.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; 
+&lt;InlineUIContainer&gt;&lt;Button Content='Implant Removal' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+The Town player may try to remove this implant from a defeated Alien controlled townsperson, thus breaking the Alien player's control.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Removing the implant generates an electric shock may erases all memory of the Alien HQ from the victim's memory, a unique safegard which is built into the implant's circuits.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Click a flashing space to begin.</t>
+  </si>
+  <si>
     <t>&lt;Bold&gt;e012t Interrogations&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r8.7.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Any conscious, defeated, Alien controlled counter may be interrogated by a Town controlled piece. Choose a building area that is not colored black. If Zebulon is found, the counter is placed on the board and can be defeated in combat to win the game. 
+Any conscious, defeated, Alien controlled counter may be interrogated by a Town controlled piece. Click on flashing space to begin. Select OK button in helper panel.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Choose a building area that is not colored black. If Zebulon is found, the counter is placed on the board and can be defeated in combat to win the game. 
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
 Click a flashing space to begin.
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
@@ -797,7 +799,7 @@
         <v>14</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="45" x14ac:dyDescent="0.25">
@@ -821,7 +823,7 @@
         <v>17</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="240" x14ac:dyDescent="0.25">
@@ -829,7 +831,7 @@
         <v>21</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="75" x14ac:dyDescent="0.25">
@@ -845,15 +847,15 @@
         <v>27</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="120" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>49</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -893,18 +895,18 @@
         <v>36</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" ht="120" x14ac:dyDescent="0.25">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>34</v>
       </c>
@@ -914,18 +916,18 @@
     </row>
     <row r="22" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -933,7 +935,7 @@
         <v>39</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>41</v>
+        <v>54</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="30" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
fixed up rules and events
</commit_message>
<xml_diff>
--- a/DesignDocs/Events.xlsx
+++ b/DesignDocs/Events.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstewa01\source\repos\happysulla\TheyveInvadedPleasantville\DesignDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{332CFE25-C099-4B4E-90C2-6D8A6D07304A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3B42CC6F-CDCD-4E0B-B3E9-E79F6847BC35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="90" windowWidth="29040" windowHeight="15510" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
+    <workbookView xWindow="28680" yWindow="90" windowWidth="29040" windowHeight="16230" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
   </bookViews>
   <sheets>
     <sheet name="Events" sheetId="1" r:id="rId1"/>
@@ -172,27 +172,6 @@
     <t>e011t</t>
   </si>
   <si>
-    <t>&lt;Bold&gt;e010t Influences&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r7.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Influencing is how the Town player convinces other uncontrolled townspeople to join their side. Click a flashing space to start a influence process.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-To influence another uncontrolled counter, the Town player compares the Influence Factors (bottom right per &lt;InlineUIContainer&gt;&lt;Button Content='r2.2.4' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;) and compares the odds ration to the 
-&lt;InlineUIContainer&gt;&lt;Button Content='Influence Results' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table adjusting with the 
-&lt;InlineUIContainer&gt;&lt;Button Content='Influence Modifiers' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-After completion of all possible infleunces have occurred, the game automatically moves to the Combat phase.</t>
-  </si>
-  <si>
-    <t>&lt;Bold&gt;e009t Conversations&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r7.1' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Conversation is how the Town player discovers if a townsperson is Alien controlled.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Click a flashing space to start a conversation.&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-On a roll of nine or better including modifiers from the &lt;InlineUIContainer&gt;&lt;Button Content='Conversation Modifiers' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table, the Town player deteremines if it is Alien controlled counter.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-After completion of all possible conversations, the game automatically moves to the Influence phase.</t>
-  </si>
-  <si>
     <t>e012t</t>
   </si>
   <si>
@@ -233,16 +212,6 @@
     <t>e013t</t>
   </si>
   <si>
-    <t>&lt;Bold&gt;e011t Combats&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r8.0' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-All combat is voluntary. Combat is started by clicking a flashing red space. If the Town player attacks one or more uncontrolled counters thinking them to be Alien controlled, the result is automatically 'Attacker Wins' for the Town player, regardless of the number of uncontrolled townspeople. 
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-The Combat Factors &lt;InlineUIContainer&gt;&lt;Button Content='r2.2.5' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; are compared to arriving at a postive difference (attacker is always greater number). The &lt;InlineUIContainer&gt;&lt;Button Content='Combat Results' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table determines the outcome.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;Combat can be skipped by clicking the following image.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-                                        &lt;InlineUIContainer&gt;&lt;Image Name='Continue011t' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
-  </si>
-  <si>
     <t>&lt;Bold&gt;e005 Random Movement&lt;/Bold&gt; &lt;InlineUIContainer&gt;&lt;Button Content='r6.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
 Four townspeople move randomly in any given turn. The &lt;InlineUIContainer&gt;&lt;Button Content='Townspeople' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table determines who moves. The destination is per the 
@@ -376,6 +345,36 @@
 Click a flashing space to begin.
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
                 &lt;InlineUIContainer&gt;&lt;Image Name='Interrogation' Height='180' Width='300'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e010t Influences&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r7.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Influencing is how the Town player convinces other uncontrolled townspeople to join their side. Click a flashing space to start an influence attempt. 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+To influence another uncontrolled counter, the Town player compares the Influence Factors (bottom right per &lt;InlineUIContainer&gt;&lt;Button Content='r2.2.4' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;) and compares the odds ratio to the 
+&lt;InlineUIContainer&gt;&lt;Button Content='Influence Results' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table adjusting with the 
+&lt;InlineUIContainer&gt;&lt;Button Content='Influence Modifiers' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+After completion of all possible infleunces have occurred, the game automatically moves to the Combat phase. All flashing spaces must be chosen. Select &lt;Bold&gt;Cancel&lt;/Bold&gt; button if want to skip influence attempt.</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e009t Conversations&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r7.1' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Conversation is how the Town player discovers if a townsperson is Alien controlled. Click a flashing space to start a conversation.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+On a roll of nine or better including modifiers from the &lt;InlineUIContainer&gt;&lt;Button Content='Conversation Modifiers' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table, the Town player deteremines if it is Alien controlled counter.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+After completion of all possible conversations, the game automatically moves to the Influence phase. All flashing spaces must be chosen. Select &lt;Bold&gt;Cancel&lt;/Bold&gt; button if want to skip conversation attempt.</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e011t Combats&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r8.0' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+All combat is voluntary. Combat is started by clicking a flashing red space. If the Town player attacks one or more uncontrolled counters thinking them to be Alien controlled, the result is automatically 'Win' for the Town player, regardless of the number of uncontrolled townspeople. 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+The Combat Factors &lt;InlineUIContainer&gt;&lt;Button Content='r2.2.5' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; are compared to arriving at a postive difference (attacker is always greater number). The &lt;InlineUIContainer&gt;&lt;Button Content='Combat Results' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table determines the outcome.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;Combat can be skipped by clicking the following image.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+                                        &lt;InlineUIContainer&gt;&lt;Image Name='Continue011t' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
   </si>
 </sst>
 </file>
@@ -751,7 +750,7 @@
         <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -799,7 +798,7 @@
         <v>14</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="45" x14ac:dyDescent="0.25">
@@ -823,7 +822,7 @@
         <v>17</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="240" x14ac:dyDescent="0.25">
@@ -831,7 +830,7 @@
         <v>21</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="75" x14ac:dyDescent="0.25">
@@ -847,15 +846,15 @@
         <v>27</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="120" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -863,15 +862,15 @@
         <v>29</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" ht="150" x14ac:dyDescent="0.25">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="165" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>30</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>32</v>
+        <v>53</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="165" x14ac:dyDescent="0.25">
@@ -879,63 +878,63 @@
         <v>31</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>40</v>
+        <v>55</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B18" s="2" t="s">
         <v>35</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B22" s="2" t="s">
         <v>42</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B23" s="2" t="s">
         <v>43</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="120" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="30" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
working on changing Takeover processes
</commit_message>
<xml_diff>
--- a/DesignDocs/Events.xlsx
+++ b/DesignDocs/Events.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstewa01\source\repos\happysulla\TheyveInvadedPleasantville\DesignDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3B42CC6F-CDCD-4E0B-B3E9-E79F6847BC35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3E398438-0DD9-4CE1-8579-9759C0F065D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="90" windowWidth="29040" windowHeight="16230" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
   </bookViews>
@@ -326,25 +326,14 @@
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;</t>
   </si>
   <si>
-    <t>&lt;Bold&gt;e013t Implant Removals&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r8.7.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; 
-&lt;InlineUIContainer&gt;&lt;Button Content='Implant Removal' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-The Town player may try to remove this implant from a defeated Alien controlled townsperson, thus breaking the Alien player's control.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Removing the implant generates an electric shock may erases all memory of the Alien HQ from the victim's memory, a unique safegard which is built into the implant's circuits.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Click a flashing space to begin.</t>
-  </si>
-  <si>
-    <t>&lt;Bold&gt;e012t Interrogations&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r8.7.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Any conscious, defeated, Alien controlled counter may be interrogated by a Town controlled piece. Click on flashing space to begin. Select OK button in helper panel.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Choose a building area that is not colored black. If Zebulon is found, the counter is placed on the board and can be defeated in combat to win the game. 
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Click a flashing space to begin.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-                &lt;InlineUIContainer&gt;&lt;Image Name='Interrogation' Height='180' Width='300'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+    <t>&lt;Bold&gt;e011t Combats&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r8.0' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+All combat is voluntary. Combat is started by clicking a flashing red space. If the Town player attacks one or more uncontrolled counters thinking them to be Alien controlled, the result is automatically 'Win' for the Town player, regardless of the number of uncontrolled townspeople. 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+The Combat Factors &lt;InlineUIContainer&gt;&lt;Button Content='r2.2.5' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; are compared to arriving at a postive difference (attacker is always greater number). The &lt;InlineUIContainer&gt;&lt;Button Content='Combat Results' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table determines the outcome.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;Combat can be skipped by clicking the following image.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+                                        &lt;InlineUIContainer&gt;&lt;Image Name='Continue011t' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
   </si>
   <si>
     <t>&lt;Bold&gt;e010t Influences&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r7.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
@@ -355,7 +344,7 @@
 &lt;InlineUIContainer&gt;&lt;Button Content='Influence Results' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table adjusting with the 
 &lt;InlineUIContainer&gt;&lt;Button Content='Influence Modifiers' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;.
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
-After completion of all possible infleunces have occurred, the game automatically moves to the Combat phase. All flashing spaces must be chosen. Select &lt;Bold&gt;Cancel&lt;/Bold&gt; button if want to skip influence attempt.</t>
+After completion of all possible infleunces have occurred, the game automatically moves to the Combat phase. All flashing spaces must be chosen. Each flashing space must be visited. If you want to skip the space, select &lt;Bold&gt;Cancel&lt;/Bold&gt; button when it appears after clicking the flashing space..</t>
   </si>
   <si>
     <t>&lt;Bold&gt;e009t Conversations&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r7.1' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
@@ -364,17 +353,28 @@
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
 On a roll of nine or better including modifiers from the &lt;InlineUIContainer&gt;&lt;Button Content='Conversation Modifiers' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table, the Town player deteremines if it is Alien controlled counter.
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
-After completion of all possible conversations, the game automatically moves to the Influence phase. All flashing spaces must be chosen. Select &lt;Bold&gt;Cancel&lt;/Bold&gt; button if want to skip conversation attempt.</t>
-  </si>
-  <si>
-    <t>&lt;Bold&gt;e011t Combats&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r8.0' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-All combat is voluntary. Combat is started by clicking a flashing red space. If the Town player attacks one or more uncontrolled counters thinking them to be Alien controlled, the result is automatically 'Win' for the Town player, regardless of the number of uncontrolled townspeople. 
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-The Combat Factors &lt;InlineUIContainer&gt;&lt;Button Content='r2.2.5' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; are compared to arriving at a postive difference (attacker is always greater number). The &lt;InlineUIContainer&gt;&lt;Button Content='Combat Results' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table determines the outcome.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;Combat can be skipped by clicking the following image.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-                                        &lt;InlineUIContainer&gt;&lt;Image Name='Continue011t' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+After completion of all possible conversations, the game automatically moves to the Influence phase. All flashing spaces must be chosen. Each flashing space must be visited. If you want to skip the space, select &lt;Bold&gt;Cancel&lt;/Bold&gt; button when it appears after clicking the flashing space..</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e012t Interrogations&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r8.7.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Any conscious, defeated, Alien controlled counter may be interrogated by a Town controlled piece. Click on flashing space to begin. Select OK button in helper panel.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Choose a building area that is not colored black. If Zebulon is found, the counter is placed on the board and can be defeated in combat to win the game. 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Click a flashing space to begin. Each flashing space must be visited. If you want to skip the space, select &lt;Bold&gt;Cancel&lt;/Bold&gt; button when it appears after clicking the flashing space.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+                &lt;InlineUIContainer&gt;&lt;Image Name='Interrogation' Height='180' Width='300'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e013t Implant Removals&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r8.7.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; 
+&lt;InlineUIContainer&gt;&lt;Button Content='Implant Removal' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+The Town player may try to remove this implant from a defeated Alien controlled townsperson, thus breaking the Alien player's control.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Removing the implant generates an electric shock may erases all memory of the Alien HQ from the victim's memory, a unique safegard which is built into the implant's circuits. Each flashing space must be visited. If you want to skip the space (for example to allow interrogation to happen prior to implant removal), select &lt;Bold&gt;Cancel&lt;/Bold&gt; button when it appears after clicking the flashing space.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Click a flashing space to begin.</t>
   </si>
 </sst>
 </file>
@@ -862,7 +862,7 @@
         <v>29</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="165" x14ac:dyDescent="0.25">
@@ -870,7 +870,7 @@
         <v>30</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="165" x14ac:dyDescent="0.25">
@@ -878,7 +878,7 @@
         <v>31</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="75" x14ac:dyDescent="0.25">
@@ -910,7 +910,7 @@
         <v>32</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="75" x14ac:dyDescent="0.25">
@@ -929,12 +929,12 @@
         <v>43</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="120" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" ht="150" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>37</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="30" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Fix recover of Takeover and last turn
</commit_message>
<xml_diff>
--- a/DesignDocs/Events.xlsx
+++ b/DesignDocs/Events.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstewa01\source\repos\happysulla\TheyveInvadedPleasantville\DesignDocs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstew\source\repos\TheyveInvadedPleasantville\DesignDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3E398438-0DD9-4CE1-8579-9759C0F065D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DD2BF702-FFB5-4462-A0D8-FB3B678C13FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="90" windowWidth="29040" windowHeight="16230" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
   </bookViews>
   <sheets>
     <sheet name="Events" sheetId="1" r:id="rId1"/>
@@ -336,6 +336,28 @@
                                         &lt;InlineUIContainer&gt;&lt;Image Name='Continue011t' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
   </si>
   <si>
+    <t>&lt;Bold&gt;e012t Interrogations&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r8.7.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Any conscious, defeated, Alien controlled counter may be interrogated by a Town controlled piece. Click on flashing space to begin. Select OK button in helper panel.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Choose a building area that is not colored black. If Zebulon is found, the counter is placed on the board and can be defeated in combat to win the game. 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Click a flashing space to begin. Each flashing space must be visited. If you want to skip the space, select &lt;Bold&gt;Cancel&lt;/Bold&gt; button when it appears after clicking the flashing space.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+                &lt;InlineUIContainer&gt;&lt;Image Name='Interrogation' Height='180' Width='300'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e009t Conversations&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r7.1' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Conversation is how the Town player discovers if a townsperson is Alien controlled. Click a flashing space to start a conversation.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+On a roll of nine or better including modifiers from the &lt;InlineUIContainer&gt;&lt;Button Content='Conversation Modifiers' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table, the Town player deteremines if it is Alien controlled counter.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+After completion of all possible conversations, the game automatically moves to the Influence phase. 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+All flashing spaces must be clicked. If you want to skip a space, select &lt;Bold&gt;Cancel&lt;/Bold&gt; button when it appears after clicking the flashing space.</t>
+  </si>
+  <si>
     <t>&lt;Bold&gt;e010t Influences&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r7.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
 Influencing is how the Town player convinces other uncontrolled townspeople to join their side. Click a flashing space to start an influence attempt. 
@@ -344,27 +366,9 @@
 &lt;InlineUIContainer&gt;&lt;Button Content='Influence Results' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table adjusting with the 
 &lt;InlineUIContainer&gt;&lt;Button Content='Influence Modifiers' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;.
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
-After completion of all possible infleunces have occurred, the game automatically moves to the Combat phase. All flashing spaces must be chosen. Each flashing space must be visited. If you want to skip the space, select &lt;Bold&gt;Cancel&lt;/Bold&gt; button when it appears after clicking the flashing space..</t>
-  </si>
-  <si>
-    <t>&lt;Bold&gt;e009t Conversations&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r7.1' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Conversation is how the Town player discovers if a townsperson is Alien controlled. Click a flashing space to start a conversation.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-On a roll of nine or better including modifiers from the &lt;InlineUIContainer&gt;&lt;Button Content='Conversation Modifiers' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table, the Town player deteremines if it is Alien controlled counter.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-After completion of all possible conversations, the game automatically moves to the Influence phase. All flashing spaces must be chosen. Each flashing space must be visited. If you want to skip the space, select &lt;Bold&gt;Cancel&lt;/Bold&gt; button when it appears after clicking the flashing space..</t>
-  </si>
-  <si>
-    <t>&lt;Bold&gt;e012t Interrogations&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r8.7.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Any conscious, defeated, Alien controlled counter may be interrogated by a Town controlled piece. Click on flashing space to begin. Select OK button in helper panel.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Choose a building area that is not colored black. If Zebulon is found, the counter is placed on the board and can be defeated in combat to win the game. 
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Click a flashing space to begin. Each flashing space must be visited. If you want to skip the space, select &lt;Bold&gt;Cancel&lt;/Bold&gt; button when it appears after clicking the flashing space.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-                &lt;InlineUIContainer&gt;&lt;Image Name='Interrogation' Height='180' Width='300'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+After completion of all possible infleunces have occurred, the game automatically moves to the Combat phase. 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+All flashing spaces must be clicked. If you want to skip a space, select &lt;Bold&gt;Cancel&lt;/Bold&gt; button when it appears after clicking the flashing space.</t>
   </si>
   <si>
     <t>&lt;Bold&gt;e013t Implant Removals&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r8.7.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; 
@@ -372,7 +376,9 @@
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
 The Town player may try to remove this implant from a defeated Alien controlled townsperson, thus breaking the Alien player's control.
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Removing the implant generates an electric shock may erases all memory of the Alien HQ from the victim's memory, a unique safegard which is built into the implant's circuits. Each flashing space must be visited. If you want to skip the space (for example to allow interrogation to happen prior to implant removal), select &lt;Bold&gt;Cancel&lt;/Bold&gt; button when it appears after clicking the flashing space.
+Removing the implant generates an electric shock may erases all memory of the Alien HQ from the victim's memory, a unique safegard which is built into the implant's circuits. 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+All flashing spaces must be clicked. If you want to skip the space (for example to allow interrogation to happen prior to implant removal), select &lt;Bold&gt;Cancel&lt;/Bold&gt; button when it appears after clicking the flashing space.
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
 Click a flashing space to begin.</t>
   </si>
@@ -857,7 +863,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="135" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" ht="150" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>29</v>
       </c>
@@ -865,12 +871,12 @@
         <v>53</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="165" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" ht="180" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>30</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="165" x14ac:dyDescent="0.25">
@@ -910,7 +916,7 @@
         <v>32</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="75" x14ac:dyDescent="0.25">
@@ -929,7 +935,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="150" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" ht="165" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>37</v>
       </c>

</xml_diff>